<commit_message>
i18n: remove all Russian text and ruble amounts from public-facing files
examples/ fixtures (requirements_wallet.docx, example_test_cases.xlsx,
README.md) are now fully English with USD amounts — this is the
international version of the repo, and the fixtures need to read cleanly
for a non-Russian reviewer without needing translation.

SKILL.md's description dropped the literal Cyrillic trigger phrases; the
skill still handles requests phrased in other languages, that behavior
just isn't spelled out with example Cyrillic text anymore. The 'Раздел ТЗ'
example column name in Phase 2 became 'Spec Section'.

test_design.md's ruble example amounts became dollar amounts.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYfZkPnWEHmFmb45hkqkyv
</commit_message>
<xml_diff>
--- a/examples/example_test_cases.xlsx
+++ b/examples/example_test_cases.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Тест-кейсы" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -427,12 +427,12 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
-    <col width="52" customWidth="1" min="5" max="5"/>
-    <col width="52" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -444,42 +444,42 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Раздел</t>
+          <t>Section</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Заголовок</t>
+          <t>Title</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Предусловия</t>
+          <t>Preconditions</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Шаги</t>
+          <t>Steps</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Ожидаемый результат</t>
+          <t>Expected Result</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Приоритет</t>
+          <t>Priority</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Тип</t>
+          <t>Type</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Автотест</t>
+          <t>Automated</t>
         </is>
       </c>
     </row>
@@ -491,30 +491,30 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Авторизация</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Вход по корректному паролю</t>
+          <t>Sign in with the correct password</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Пользователь зарегистрирован, статус подтверждён</t>
+          <t>User is registered, status is verified</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>1. Открыть экран входа
-2. Ввести номер +79001112233
-3. Ввести пароль Qwerty123!
-4. Нажать «Войти»</t>
+          <t>1. Open the sign-in screen
+2. Enter phone +14155550112
+3. Enter password Qwerty123!
+4. Tap “Sign in”</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Открывается главный экран, в шапке отображается баланс кошелька</t>
+          <t>The home screen opens, the wallet balance is shown in the header</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -524,12 +524,12 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Позитивный</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -541,30 +541,30 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Авторизация</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Вход с неверным паролем</t>
+          <t>Sign in with an incorrect password</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Пользователь зарегистрирован</t>
+          <t>User is registered</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>1. Открыть экран входа
-2. Ввести номер +79001112233
-3. Ввести пароль Qwerty000
-4. Нажать «Войти»</t>
+          <t>1. Open the sign-in screen
+2. Enter phone +14155550112
+3. Enter password Qwerty000
+4. Tap “Sign in”</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Показывается сообщение «Неверный логин или пароль», переход на главный экран не происходит</t>
+          <t>The message “Incorrect login or password” is shown, no transition to the home screen occurs</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -574,12 +574,12 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Негативный</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -591,29 +591,29 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Профиль</t>
+          <t>Profile</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Смена номера телефона без подтверждения кодом</t>
+          <t>Change phone number without SMS confirmation</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Пользователь авторизован, открыт раздел «Профиль»</t>
+          <t>User is signed in, the Profile section is open</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>1. Нажать «Изменить номер»
-2. Ввести новый номер +79004445566
-3. Нажать «Сохранить», не вводя код из SMS</t>
+          <t>1. Tap “Change number”
+2. Enter new number +14155550199
+3. Tap “Save” without entering the SMS code</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Номер не сохраняется, поле кода подсвечено красным с текстом «Введите код из SMS»</t>
+          <t>The number is not saved, the code field is highlighted in red with the text “Enter the SMS code”</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -623,12 +623,12 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Негативный</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>No</t>
         </is>
       </c>
     </row>

</xml_diff>